<commit_message>
OLX 6m+ Recherche - neues Sheet + Eintraege ergaenzt
Live-Suche auf OLX.pt nach Jurten mit min. 6 m Durchmesser:

3 konkrete Funde >=6m identifiziert:
1. Yurts mongois (Igreja Nova/Cheleiros, Mafra) - 6m / 28m2 / 5.000 EUR
   gebraucht, klassisch mongolisch (Filz), Pelletofen optional
2. Tenda Yurt Original Quirguistao (Palmela, Setubal) - ca. 6m / 28m2
   neu/authentisch, Marke Yourta 'Serenity', vollstaendige Originaldeko
3. Yurt Made in Portugal (Loures) - 6m / 28m2 / 8.400 EUR
   neuer PT-Hersteller seit 2020, auch 5m/7m/8m verfuegbar

Ausgeschlossen: Mafra-Angebot (nur 5,5m).

Neuer PT-Hersteller "Yurt Made in Portugal" auch zu Sheet "Hersteller
Neu" hinzugefuegt (5m=6.900 / 6m=8.400 / 7-8m Anfrage).

Sheet 2 (Gebrauchtmarkt) um 2 konkrete OLX-Direktlinks ergaenzt.

https://claude.ai/code/session_01Wo6qsEhTrQuYRViomLojPq
</commit_message>
<xml_diff>
--- a/Jurten_Recherche_Algarve.xlsx
+++ b/Jurten_Recherche_Algarve.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Top 5 Empfehlungen" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Hinweise" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Casa dos Sonhos Detail" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="OLX 6m+ Funde" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +48,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="4">
@@ -95,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -113,6 +118,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1812,102 +1820,154 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Yurt Workshop UK</t>
+          <t>Yurt Made in Portugal (Loures, ueber OLX)</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Portugal (Loures, Lisboa)</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>https://www.yurtworkshop.com/</t>
+          <t>https://www.olx.pt/d/anuncio/yurt-made-in-portugal-IDIyzPL.html</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>5-7m</t>
+          <t>5m=20m2 / 6m=28m2 / 7-8m auf Anfrage</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Anfrage GBP/EUR</t>
+          <t>5m 6.900 / 6m 8.400 / 7-8m Anfrage</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Eichen-/Kastanien-Holz + Canvas + Wollfilz</t>
+          <t>Holz + Filz + Plane (modern), portugiesisch handgefertigt</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Mittel - Brexit-Zoll Aufschlag</t>
+          <t>Sehr gut - lokaler PT-Hersteller seit 2020, kein Import-Zoll/IVA</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>UK-&gt;PT 1.500-2.500 EUR + EU-Zoll/IVA bei Brexit-Import</t>
+          <t>Innerhalb PT - Lieferung+Aufbau EXTRA (standortabhaengig)</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Etabliert; Brexit verteuert Lieferung in EU erheblich</t>
+          <t>Neuer kleiner PT-Hersteller bei Lissabon, 'modern take on ancient living'. OLX-Praesenz seit 2020.</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>9.000-13.000</t>
+          <t>8.400-10.500 inkl. Aufbau (6m)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Yurt Workshop UK</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.yurtworkshop.com/</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>5-7m</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Anfrage GBP/EUR</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Eichen-/Kastanien-Holz + Canvas + Wollfilz</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Mittel - Brexit-Zoll Aufschlag</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>UK-&gt;PT 1.500-2.500 EUR + EU-Zoll/IVA bei Brexit-Import</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Etabliert; Brexit verteuert Lieferung in EU erheblich</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>9.000-13.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
           <t>FamWest</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>https://www.famwest.de/en/mongolian-yurts/</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>5-9m Durchmesser</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>Anfrage</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Filz + Canvas</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Mittel</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>DE-&gt;PT 1.500-2.000 EUR</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>5/6/7/8/9 m Optionen, inkl 19% MwSt</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>ca. 6.000-15.000</t>
         </is>
@@ -1924,7 +1984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2123,64 +2183,62 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Kleinanzeigen - Jurte Suche</t>
+          <t>OLX PT: Yurts mongois (Igreja Nova/Cheleiros, Mafra)</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>kleinanzeigen.de</t>
+          <t>olx.pt</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Deutschland weit</t>
+          <t>PT - Mafra (bei Lissabon)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>diverse</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>1.000-15.000</t>
-        </is>
+          <t>28 m2 (6 m Durchmesser)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>5000</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Neu bis stark gebraucht</t>
+          <t>Gebraucht / Restposten</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>https://www.kleinanzeigen.de/s-jurte/k0</t>
+          <t>https://www.olx.pt/d/anuncio/yurts-mongis-mongolian-yurts-IDHQ8sJ.html</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Ja - Spedition 500-1.500 EUR</t>
+          <t>Ja - inland PT, Transport+Aufbau gegen Aufpreis</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Marktplatz, wechselnde Angebote, regelmaessig pruefen</t>
+          <t>BESTPREIS 6m+ auf OLX! Filzdecke (warm/kuehl), mobile Aufbau auf jeder ebenen Flaeche. Optional Pelletofen gegen Aufpreis. Direkt vom Verkaeufer.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>eBay.de Jurten Kategorie</t>
+          <t>Kleinanzeigen - Jurte Suche</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>eBay.de</t>
+          <t>kleinanzeigen.de</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Deutschland weit</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2190,44 +2248,44 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>200-10.000+</t>
+          <t>1.000-15.000</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Neu/gebraucht</t>
+          <t>Neu bis stark gebraucht</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>https://www.ebay.de/b/Jurte-Zelt/bn_7005694261</t>
+          <t>https://www.kleinanzeigen.de/s-jurte/k0</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Versand variiert</t>
+          <t>Ja - Spedition 500-1.500 EUR</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Auch Pfadfinder-Jurten (gross, billig, aber Plane nicht UV-fest)</t>
+          <t>Marktplatz, wechselnde Angebote, regelmaessig pruefen</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>eBay.co.uk Yurt</t>
+          <t>eBay.de Jurten Kategorie</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>eBay UK</t>
+          <t>eBay.de</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -2237,54 +2295,54 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>1.500-12.000</t>
+          <t>200-10.000+</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Gebraucht</t>
+          <t>Neu/gebraucht</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>https://www.ebay.co.uk/sch/i.html?_nkw=yurt</t>
+          <t>https://www.ebay.de/b/Jurte-Zelt/bn_7005694261</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Ja - Brexit-Zoll bei Import nach PT (~7% Zoll + 23% IVA)</t>
+          <t>Versand variiert</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Brexit verteuert UK-Importe stark</t>
+          <t>Auch Pfadfinder-Jurten (gross, billig, aber Plane nicht UV-fest)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>LeBonCoin Yourte</t>
+          <t>eBay.co.uk Yurt</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>leboncoin.fr</t>
+          <t>eBay UK</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Frankreich (variable)</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>10-50 m2</t>
+          <t>diverse</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1.500-20.000</t>
+          <t>1.500-12.000</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -2294,44 +2352,44 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>https://www.leboncoin.fr/ck/ventes_immobilieres/yourte</t>
+          <t>https://www.ebay.co.uk/sch/i.html?_nkw=yurt</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Ja - Spedition FR-&gt;PT 800-1.500 EUR</t>
+          <t>Ja - Brexit-Zoll bei Import nach PT (~7% Zoll + 23% IVA)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Beispiel: 6m yourte mit Wollisolierung gelistet</t>
+          <t>Brexit verteuert UK-Importe stark</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Wallapop Yurtas</t>
+          <t>LeBonCoin Yourte</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>wallapop.com</t>
+          <t>leboncoin.fr</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>Frankreich (variable)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>diverse</t>
+          <t>10-50 m2</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>5.000-25.000</t>
+          <t>1.500-20.000</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -2341,29 +2399,29 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>https://es.wallapop.com/muebles-deco-y-jardin/yurtas</t>
+          <t>https://www.leboncoin.fr/ck/ventes_immobilieres/yourte</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Ja - ES-&gt;PT guenstig 500-1.000 EUR</t>
+          <t>Ja - Spedition FR-&gt;PT 800-1.500 EUR</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>9 Eintraege typischerweise gelistet</t>
+          <t>Beispiel: 6m yourte mit Wollisolierung gelistet</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Milanuncios Yurta</t>
+          <t>Wallapop Yurtas</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>milanuncios.com</t>
+          <t>wallapop.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -2373,59 +2431,59 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>diverse 40-80 m2</t>
+          <t>diverse</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>22.500-42.000</t>
+          <t>5.000-25.000</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Neu/gebraucht</t>
+          <t>Gebraucht</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>https://www.milanuncios.com/anuncios/yurt-yurta.htm</t>
+          <t>https://es.wallapop.com/muebles-deco-y-jardin/yurtas</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja - ES-&gt;PT guenstig 500-1.000 EUR</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Komplett ausgestattet 27.500 EUR, ohne Moebel 22.500 EUR (Beispiel)</t>
+          <t>9 Eintraege typischerweise gelistet</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>OLX Portugal yurts</t>
+          <t>Milanuncios Yurta</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>olx.pt</t>
+          <t>milanuncios.com</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Spanien</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>diverse</t>
+          <t>diverse 40-80 m2</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>variabel</t>
+          <t>22.500-42.000</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -2435,86 +2493,86 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>https://www.olx.pt/moveis-casa-e-jardim/q-yurts/</t>
+          <t>https://www.milanuncios.com/anuncios/yurt-yurta.htm</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Ja - innerhalb PT</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>INLAND PT - keine Zoll, kein Auslandsversand</t>
+          <t>Komplett ausgestattet 27.500 EUR, ohne Moebel 22.500 EUR (Beispiel)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Yurt Workshop Secondhand</t>
+          <t>OLX Portugal yurts (Kategorie-Uebersicht)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>yurtworkshop.com (Spanien)</t>
+          <t>olx.pt</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Spanien Granada</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>5-7m</t>
+          <t>diverse</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>3.000-10.000</t>
+          <t>variabel</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Gebraucht (vom Hersteller)</t>
+          <t>Neu/gebraucht</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>https://www.yurtworkshop.com/Buy_Your_Yurt/Second-Hand-Yurts-For-Sale.html</t>
+          <t>https://www.olx.pt/moveis-casa-e-jardim/jardim-e-bricolage/q-yurts/</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Ja - ES-&gt;PT 600-1.200 EUR</t>
+          <t>Ja - innerhalb PT</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Vom Hersteller selbst - Qualitaet gepruef</t>
+          <t>INLAND PT - keine Zoll, kein Auslandsversand</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Casa Dos Sonhos Secondhand</t>
+          <t>OLX PT: Tenda Yurt Original Quirguistao (Palmela)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Facebook Casa Dos Sonhos</t>
+          <t>olx.pt</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Portugal (Alentejo)</t>
+          <t>PT - Palmela (Setubal)</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>28 m2 (ca. 6 m Durchmesser, 30 Personen)</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -2524,133 +2582,133 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Gebraucht direkt vom Eigentuemer</t>
+          <t>Neu/handgefertigt (Originalimport Issyk-Kul Quirguistao)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/yurtscasadossonhos/posts/3660919220624833/</t>
+          <t>https://www.olx.pt/d/anuncio/tenda-yurt-original-do-quirguisto-yurt-tent-original-from-kyrgystan-IDHEwz9.html</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Ja - inland PT</t>
+          <t>Ja - PT-inland, Versand EXTRA (Region Lissabon)</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Hersteller direkt, ggf. Garantie</t>
+          <t>Marke 'Yourta', Modell 'Serenity'. Komplette Originalausstattung: Schilf-Geflecht, Wolle/Filz, Shyrdak-Teppich, Baskur-Band, Korpe-Kissen, geschnitzte Holztuer. Hand-Applikation. Keine Baugenehmigung noetig.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Yurt Market (worldwide)</t>
+          <t>Yurt Workshop Secondhand</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>yurtmarket.com</t>
+          <t>yurtworkshop.com (Spanien)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>Spanien Granada</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>diverse</t>
+          <t>5-7m</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>variabel</t>
+          <t>3.000-10.000</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Neu/gebraucht</t>
+          <t>Gebraucht (vom Hersteller)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>https://www.yurtmarket.com/</t>
+          <t>https://www.yurtworkshop.com/Buy_Your_Yurt/Second-Hand-Yurts-For-Sale.html</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Versand variiert je Anbieter</t>
+          <t>Ja - ES-&gt;PT 600-1.200 EUR</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Welt-Marktplatz</t>
+          <t>Vom Hersteller selbst - Qualitaet gepruef</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Yurt Forum Classifieds</t>
+          <t>Casa Dos Sonhos Secondhand</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>yurtforum.com</t>
+          <t>Facebook Casa Dos Sonhos</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>Portugal (Alentejo)</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>diverse</t>
+          <t>5m</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>variabel</t>
+          <t>Anfrage</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Gebraucht</t>
+          <t>Gebraucht direkt vom Eigentuemer</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>https://www.yurtforum.com/classifieds/</t>
+          <t>https://www.facebook.com/yurtscasadossonhos/posts/3660919220624833/</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Versand variiert</t>
+          <t>Ja - inland PT</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Community-Marktplatz, oft USA-fokussiert</t>
+          <t>Hersteller direkt, ggf. Garantie</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Groovy Yurts Clearance</t>
+          <t>Yurt Market (worldwide)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>groovyyurts.com</t>
+          <t>yurtmarket.com</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Kanada/USA</t>
+          <t>International</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -2660,72 +2718,166 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>USD 2.790-18.950</t>
+          <t>variabel</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Restposten/leicht gebraucht</t>
+          <t>Neu/gebraucht</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>https://www.groovyyurts.com/catalogue-clearance-and-sale</t>
+          <t>https://www.yurtmarket.com/</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Nein - hauptsaechlich Nordamerika; Versand teuer</t>
+          <t>Versand variiert je Anbieter</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Eher fuer US/CA - hohe Versandkosten nach EU/PT</t>
+          <t>Welt-Marktplatz</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
+          <t>Yurt Forum Classifieds</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>yurtforum.com</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>diverse</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>variabel</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Gebraucht</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.yurtforum.com/classifieds/</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Versand variiert</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Community-Marktplatz, oft USA-fokussiert</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Groovy Yurts Clearance</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>groovyyurts.com</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Kanada/USA</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>diverse</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>USD 2.790-18.950</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Restposten/leicht gebraucht</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.groovyyurts.com/catalogue-clearance-and-sale</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Nein - hauptsaechlich Nordamerika; Versand teuer</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Eher fuer US/CA - hohe Versandkosten nach EU/PT</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>Facebook Marketplace EU</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>facebook.com/marketplace</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Diverse EU</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>diverse</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>variabel</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Gebraucht</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>https://www.facebook.com/marketplace/category/search/?query=yurt</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>Regional pruefen</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Lokale Suche pro Land empfohlen</t>
         </is>
@@ -4811,4 +4963,252 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Titel/Listing</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Standort PT</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Durchmesser</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Innenflaeche m2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Preis EUR</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Zustand</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Material/Bauart</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Versand/Aufbau</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Direktlink</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Anmerkungen / Bewertung Algarve</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Yurts mongois / Mongolian Yurts</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Igreja Nova e Cheleiros (Mafra, naehe Lissabon)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>6 m</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>28 m2</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Gebraucht/Restposten - direkt vom Verkaeufer</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Klassische mongolische Bauweise: Filzdecke (warm im Winter, kuehl im Sommer), Holzgitter, mobil auf jeder ebenen Flaeche aufbaubar</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>PT-inland, Transport+Aufbau gegen Aufpreis. Optional Pelletofen gegen Aufpreis.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.olx.pt/d/anuncio/yurts-mongis-mongolian-yurts-IDHQ8sJ.html</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>TOP-FUND: Gueneststes 6m-Angebot auf OLX. ABER: traditioneller Filz/Canvas ohne UV-Schutz - mit Schattennetz nachruesten (siehe Hinweise-Sheet) sonst Plane nur 2-3 Jahre Lebensdauer in Algarve. Mit Pelletofen+Aufbau realistisch 6.000-7.500 EUR Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="110" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Yurt Made in Portugal (Hersteller-Insertion auf OLX)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Loures (naehe Lissabon)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>6 m verfuegbar (auch 5m, 7m, 8m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ca. 28 m2 (6m)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>8400</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>NEU - Hersteller seit 2020</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Modern interpretierte traditionelle Bauweise; portugiesischer Hersteller</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Lieferung+Aufbau NICHT inklusive - extra je nach Standort und Groesse</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.olx.pt/d/anuncio/yurt-made-in-portugal-IDIyzPL.html</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Lokaler PT-Hersteller (kein Importzoll), seit 2020 aktiv. Direktkontakt ueber OLX. 5m=6.900 EUR / 6m=8.400 EUR / 7-8m auf Anfrage. Hinweis: Klimaschutz/UV-Garantie nicht spezifiziert -&gt; dringend nachfragen, ob Plane fuer Algarve geeignet ist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="110" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TENDA YURT Original do Quirguistao (Marke Yourta - Modell 'Serenity')</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Palmela (Setubal, naehe Lissabon)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ca. 6 m (geschaetzt aus 28 m2)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>28 m2 (Kapazitaet 30 Personen)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Anfrage (Region Lissabon)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Neu / handgefertigt, original aus Quirguistao (Issyk-Kul See)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Original kirgisisch: Schilf-Geflecht (Junco), Wolle und Filz. Komplette Originaldeko: Shyrdak-Teppich, Baskur-Band, Korpe-Linen-Kissen, geschnitzte Holztuer, Filz-Tuerverkleidung, dekorative Kuppelbaender</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Versand EXTRA (Region Lissabon - genauen Preis erfragen)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.olx.pt/d/anuncio/tenda-yurt-original-do-quirguisto-yurt-tent-original-from-kyrgystan-IDHEwz9.html</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>HOHE AUTHENTIZITAET: Originalimport aus Quirguistao, traditionelle Stickerei und Applikationen. PROBLEM ALGARVE: traditioneller Filz/Wolle nicht fuer 40C+ ausgelegt; Plane unter UV-Belastung anfaellig. Sehr dekorativ - eher fuer kuehlere Bergstandorte als heisse Algarve geeignet. Inserent in PT, kein Importzoll.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Ausgeschlossen (unter 6 m Mindestgroesse): 'Yurt mongol autentico Mafra' (5,5 m, 8.000 EUR) - https://www.olx.pt/d/anuncio/yurt-mongol-autntico-IDIR7sZ.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>WICHTIG: OLX-Angebote aendern sich taeglich. Vor Anfrage Live-Suche unter https://www.olx.pt/moveis-casa-e-jardim/jardim-e-bricolage/q-yurts/ pruefen. Recherche-Stand: 2026-05-11.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="A8:J8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Casa dos Sonhos Zahlungsbedingungen + Risiko-Bewertung
Bestaetigt per Facebook Messenger:
- Anzahlung sichert Termin (Teil der Gesamtsumme)
- Vollzahlung 2 Monate vor Lieferung (5/6,1/7,3m)
- Vollzahlung 3 Monate vor Lieferung (9,1m)
- 10-J. UV-Garantie auf Plane bestaetigt

ROTE FLAGGE: 100% Vorauszahlung Monate vor Lieferung ist NICHT
branchenueblich (Standard: 30-50% Anzahlung + Rest bei Abnahme).
Kaeufer traegt vollstaendiges Insolvenz- und Qualitaetsrisiko.

Mitigation-Optionen in Sheet 6 dokumentiert:
- Kreditkarte (Chargeback)
- Treuhandkonto Escrow
- Etappenzahlung verhandeln
- Persoenlicher Werkstatt-Besuch + Referenz-Telefonate VOR Vollzahlung
- Rechtsform der Firma pruefen

Social-Media-Kanaele zur Verifikation ergaenzt:
Facebook (3.617 Follower), YouTube, TikTok.

https://claude.ai/code/session_01Wo6qsEhTrQuYRViomLojPq
</commit_message>
<xml_diff>
--- a/Jurten_Recherche_Algarve.xlsx
+++ b/Jurten_Recherche_Algarve.xlsx
@@ -4253,7 +4253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B84"/>
+  <dimension ref="A1:B88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4906,7 +4906,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="30" customHeight="1">
+    <row r="65" ht="25" customHeight="1">
       <c r="A65" s="8" t="inlineStr">
         <is>
           <t>Slot-Verfuegbarkeit (Mai 2026)</t>
@@ -4914,185 +4914,233 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Atilla Berki-Style Slot-System: aktuell Dezember 2026 oder 2027 angeboten -&gt; hohe Auslastung</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="29" customHeight="1">
+          <t>Aktuell Dezember 2026 oder 2027 angeboten -&gt; hohe Auslastung</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="50" customHeight="1">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>Zahlung</t>
+          <t>Zahlungsbedingungen BESTAETIGT</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Direkt mit Hersteller, Konditionen offen (Etappenzahlung gegen Baufortschritt anfragen)</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="8" customHeight="1"/>
-    <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="5" t="inlineStr">
+          <t>1) Anzahlung sichert den Termin (Teil der Gesamtsumme). 2) VOLLZAHLUNG 2 Monate vor Lieferung (5m/6,1m/7,3m) bzw. 3 Monate vor Lieferung (9,1m). 3) Lieferung selbst KEIN Zahlungstrigger - alles vorher beglichen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="52" customHeight="1">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>RISIKO-Bewertung Zahlung</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>ROTE FLAGGE: 100% im Voraus, Monate vor Lieferung. Branchenstandard ist 30-50% Anzahlung + Restzahlung bei Abnahme. Bei CdS keinerlei Hebel mehr nach Vollzahlung. Insolvenz-/Qualitaetsrisiko liegt vollstaendig beim Kaeufer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="60" customHeight="1">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>Mitigation-Optionen</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>1) Per Kreditkarte zahlen (Chargeback-Schutz) - mit Bank vorab klaeren ob Limit reicht. 2) Treuhand-Konto (Escrow) in PT, kostet ~0,5-1% Volumen. 3) Etappenzahlung verhandeln: 30% Anzahlung / 40% bei Baustart mit Foto-/Video-Nachweis / 30% bei Abnahme vor Ort. 4) Persoenlicher Besuch+Werkstatt-Besichtigung VOR Vollzahlung erzwingen. 5) Referenzen (PT/Algarve) kontaktieren und Punkt: Termintreue+Qualitaet abfragen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="57" customHeight="1">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>Social-Media-Kanaele zur Verifikation</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Facebook https://www.facebook.com/yurtscasadossonhos/ - 3.617 Follower, regelmaessige Posts seit Jahren / YouTube https://www.youtube.com/channel/UCfenMyhVzEkX7P-lz2hjS6A - dokumentierte Aufbau-Videos / TikTok https://www.tiktok.com/@casadossonhosyurts</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="8" customHeight="1"/>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>Nachhaltigkeit / ESG</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="20" customHeight="1">
-      <c r="A69" s="8" t="inlineStr">
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="8" t="inlineStr">
         <is>
           <t>Energie Produktion</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>100% Solar in der Werkstatt</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="20" customHeight="1">
-      <c r="A70" s="8" t="inlineStr">
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="8" t="inlineStr">
         <is>
           <t>Materialien-Herkunft</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>Portugiesisch (Holz, Kork)</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="30" customHeight="1">
-      <c r="A71" s="8" t="inlineStr">
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="8" t="inlineStr">
         <is>
           <t>Soziales Engagement</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>Plant Wollverarbeitung um lokale Schafwolle aufzuwerten (Alentejo) - aktuell unterbewertet</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="8" t="inlineStr">
-        <is>
-          <t>Kreislaufwirtschaft</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>Natuerliche Materialien, kein PVC im Standard</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="8" customHeight="1"/>
-    <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="5" t="inlineStr">
-        <is>
-          <t>Risiken &amp; Hinweise</t>
         </is>
       </c>
     </row>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="8" t="inlineStr">
         <is>
+          <t>Kreislaufwirtschaft</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Natuerliche Materialien, kein PVC im Standard</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="8" customHeight="1"/>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>Risiken &amp; Hinweise</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="26" customHeight="1">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
           <t>Lieferzeit</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>Handarbeit -&gt; mehrere Monate Vorlauf einplanen</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="24" customHeight="1">
-      <c r="A76" s="8" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Handarbeit -&gt; aktuell Dezember 2026 oder 2027. Slot frueh sichern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="24" customHeight="1">
+      <c r="A79" s="8" t="inlineStr">
         <is>
           <t>Skalierung</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>Kleines Familienunternehmen - Reaktionszeit kann variieren</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="30" customHeight="1">
-      <c r="A77" s="8" t="inlineStr">
-        <is>
-          <t>Preis intransparent</t>
-        </is>
-      </c>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>Keine oeffentliche Preisliste - immer schriftliches Angebot einholen + Optionen klar definieren</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="23" customHeight="1">
-      <c r="A78" s="8" t="inlineStr">
+    <row r="80" ht="38" customHeight="1">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>HAUPTRISIKO Zahlung</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>100% Vorauszahlung 2-3 Monate vor Lieferung - vollstaendiges Kaeufer-Risiko ohne Sicherheit. Mitigation siehe Sektion 'Preis &amp; Kommerzielles'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="25" customHeight="1">
+      <c r="A81" s="8" t="inlineStr">
         <is>
           <t>Sturmkomponente</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>Algarve-Kueste: Sturm-Kit OBLIGATORISCH bestellen</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="29" customHeight="1">
-      <c r="A79" s="8" t="inlineStr">
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Algarve-Kueste: Sturm-Kit OBLIGATORISCH bestellen (Preis offen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="29" customHeight="1">
+      <c r="A82" s="8" t="inlineStr">
         <is>
           <t>Hitze Innenraum</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>Trotz 10-J. Plane: zusaetzliches Schattennetz/Pergola fuer 40C+ Sommertage empfehlenswert</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="8" customHeight="1"/>
-    <row r="81" ht="22" customHeight="1">
-      <c r="A81" s="5" t="inlineStr">
+    <row r="83" ht="53" customHeight="1">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>Verifikations-Schritte VOR Auftrag</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>1) Show-Yurt-Besuch Portalegre + Werkstatt-Tour. 2) 2 Algarve/Monchique-Referenzen telefonisch sprechen. 3) Rechtsform der Firma (Lda/Unipessoal/Einzelperson) checken. 4) Zahlungsmodalitaeten verhandeln (Etappen oder Kreditkarte).</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="8" customHeight="1"/>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t>Fazit fuer Algarve</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="54" customHeight="1">
-      <c r="A82" s="8" t="inlineStr">
+    <row r="86" ht="54" customHeight="1">
+      <c r="A86" s="8" t="inlineStr">
         <is>
           <t>Bewertung</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>TOP-EMPFEHLUNG #1 BESTAETIGT - bei 6,1m fuer 9.700 EUR all-in nicht zu schlagen, einzigartige 10-J. UV-Garantie schriftlich, lokale Produktion, Lieferung+Aufbau inkl., portugiesische Materialien, kein Import-Risiko, kein Versandstress.</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="34" customHeight="1">
-      <c r="A83" s="8" t="inlineStr">
+    <row r="87" ht="34" customHeight="1">
+      <c r="A87" s="8" t="inlineStr">
         <is>
           <t>Sweet Spot</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr">
+      <c r="B87" s="3" t="inlineStr">
         <is>
           <t>6,1m / 30 m2 zu 9.700 EUR - DEUTLICH UNTER 15k Budget, laesst Raum fuer Sturm-Kit + Kaminzug + Plattform-Vorbereitung</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="57" customHeight="1">
-      <c r="A84" s="8" t="inlineStr">
+    <row r="88" ht="57" customHeight="1">
+      <c r="A88" s="8" t="inlineStr">
         <is>
           <t>Naechster Schritt</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B88" s="3" t="inlineStr">
         <is>
           <t>Konkretes schriftliches Angebot fuer 6,1m oder 7,3m inkl. Sturm-Kit + Kaminzug + Mezzanine-Option (falls fuer 7,3m relevant) anfragen. Zahlungskonditionen klaeren (Etappenzahlung). Show-Yurt-Besuch Portalegre verhandeln. Slot 2026 bestaetigen (nicht 2027).</t>
         </is>
@@ -5102,15 +5150,15 @@
   <mergeCells count="12">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A81:B81"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A85:B85"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A77:B77"/>
     <mergeCell ref="A55:B55"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Kommunikations-Log: Atilla-Folgemail gesendet 20.05.2026
Sebastian hat die Folgemail an Atilla rausgeschickt nach seiner
Engineering-Korrektur:
- Akzeptiert Atilla's Standard-Masse (180cm Tono, jede Khaana-Spitze=Uni)
- Fragt nach Frame-only-Quote mit Atilla's Massen
- Erfragt Larch-Option, Skylight-Preis, Lieferzeit, Versand, Eigene-
  Spedition-Option, Werkstatt-Besuch

Wartet jetzt auf Atilla's Antwort (3-7 Tage erwartet).

https://claude.ai/code/session_01Wo6qsEhTrQuYRViomLojPq
</commit_message>
<xml_diff>
--- a/Jurten_Recherche_Algarve.xlsx
+++ b/Jurten_Recherche_Algarve.xlsx
@@ -7825,7 +7825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7988,12 +7988,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>~10.05.2026</t>
+          <t>20.05.2026</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Adorjan Jurta (HU)</t>
+          <t>Atilla es a Fehernep (HU)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -8003,29 +8003,29 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Adorjan</t>
+          <t>Sebastian -&gt; Atilla</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Frame-only Anfrage 8m, Larch optional, Oel-Finish, Versand PT</t>
+          <t>Akzeptiert Atilla's Engineering-Standards (180cm Tono, jede Khaana-Spitze=Uni, 2m Wand). Fragt nach: Frame-only-Quote mit Atilla's Massen, Laerche statt Buche/Kiefer, Skylight-Preis 180cm Tono, Lieferzeit, Versand frame-only Algarve, Eigene-Spedition-Option, Werkstatt-Besuch.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>✓ Teilantwort</t>
+          <t>✓ Gesendet</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Folgemail: 4 Punkte offen (Larch / Tuer-Variante / Lieferzeit / Eigener Spediteur / Werkstatt-Besuch)</t>
+          <t>Antwort abwarten (3-7 Tage). Bei Verzug nach 10 Tagen WhatsApp +36 30 657 0740.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>~10.05.2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -8040,22 +8040,22 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Adorjan -&gt; Sebastian</t>
+          <t>Sebastian -&gt; Adorjan</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>8m Rahmen 3.220.000 HUF = 8.150 EUR netto. Spezifikation Top: 48 Rafters 5x10cm, Tono 170cm 4-lagig verleimt, Wand 2m, Pinie AT Biopin-impraegniert, isolierte Tuer Standard. Versand offen.</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>Info erhalten</t>
+          <t>Frame-only Anfrage 8m, Larch optional, Oel-Finish, Versand PT</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>✓ Teilantwort</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Folge-Fragen senden</t>
+          <t>Folgemail: 4 Punkte offen (Larch / Tuer-Variante / Lieferzeit / Eigener Spediteur / Werkstatt-Besuch)</t>
         </is>
       </c>
     </row>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Versand-Spediteur wird gesucht, kein Preis. 50% Anzahlung + 50% vor Versand. Installation extra (4 Pers + Fluege + Maschinen).</t>
+          <t>8m Rahmen 3.220.000 HUF = 8.150 EUR netto. Spezifikation Top: 48 Rafters 5x10cm, Tono 170cm 4-lagig verleimt, Wand 2m, Pinie AT Biopin-impraegniert, isolierte Tuer Standard. Versand offen.</t>
         </is>
       </c>
       <c r="F7" s="16" t="inlineStr">
@@ -8092,19 +8092,19 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Folge-Fragen (Larch/Tuer/Lieferzeit) + Eigener-Spediteur-Option erfragen</t>
+          <t>Folge-Fragen senden</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>~10.05.2026</t>
+          <t>?</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Yourtetoiles &amp; Kontempobois (FR)</t>
+          <t>Adorjan Jurta (HU)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -8114,29 +8114,29 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Yourtetoiles</t>
+          <t>Adorjan -&gt; Sebastian</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Anfrage 8m Yurte</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>✓ Teilantwort</t>
+          <t>Versand-Spediteur wird gesucht, kein Preis. 50% Anzahlung + 50% vor Versand. Installation extra (4 Pers + Fluege + Maschinen).</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>Info erhalten</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>WhatsApp-Videocall Termin festlegen, beide Linien (Klassisch + Kontempo) erfragen</t>
+          <t>Folge-Fragen (Larch/Tuer/Lieferzeit) + Eigener-Spediteur-Option erfragen</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>~10.05.2026</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -8151,66 +8151,66 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Yourtetoiles -&gt; Sebastian</t>
+          <t>Sebastian -&gt; Yourtetoiles</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Empfehlen Kontempo (Holz-Rundhaus mit Zink-Dach) statt klassischer Jurte fuer Atlantik-Exposition. Devis komplett dauert noch. Bieten Visio-Call an.</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>Info erhalten</t>
+          <t>Anfrage 8m Yurte</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>✓ Teilantwort</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Visio-Call vereinbaren (3 Terminvorschlaege schicken)</t>
+          <t>WhatsApp-Videocall Termin festlegen, beide Linien (Klassisch + Kontempo) erfragen</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>~12.05.2026</t>
+          <t>?</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Casa dos Sonhos (Sarah &amp; Vladimir, PT)</t>
+          <t>Yourtetoiles &amp; Kontempobois (FR)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Facebook Messenger</t>
+          <t>E-Mail</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Sarah</t>
+          <t>Yourtetoiles -&gt; Sebastian</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Anfrage 5/6,1/7,3/9,1m Preise + Konditionen</t>
+          <t>Empfehlen Kontempo (Holz-Rundhaus mit Zink-Dach) statt klassischer Jurte fuer Atlantik-Exposition. Devis komplett dauert noch. Bieten Visio-Call an.</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>✓ Beantwortet</t>
+          <t>Info erhalten</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Visio-Call vereinbaren (3 Terminvorschlaege schicken)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>~13.05.2026</t>
+          <t>~12.05.2026</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -8225,29 +8225,29 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Sarah -&gt; Sebastian</t>
+          <t>Sebastian -&gt; Sarah</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Preise bestaetigt: 5m 7.900 / 6,1m 9.700 / 7,3m 15.750 / 9,1m 18.000 EUR delivered+erected PT. Refs Brett (Quinta Glamping) + Paula Young (verkauft 7,3m gebraucht).</t>
+          <t>Anfrage 5/6,1/7,3/9,1m Preise + Konditionen</t>
         </is>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>Quote erhalten</t>
+          <t>✓ Beantwortet</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Nachfrage NIPC/IVA/Bankdaten/Material-Spec/Vermittlung Paula</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>15.05.2026</t>
+          <t>~13.05.2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -8257,7 +8257,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>PDF Quote</t>
+          <t>Facebook Messenger</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -8267,7 +8267,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Quote 6,1m + 2.Tuer 850 + Flue-Kit 100 = 10.650 EUR. 1.000 EUR Anzahlung + 9.650 EUR am 1.8.2026. Lieferung 2. Oktoberwoche 2026.</t>
+          <t>Preise bestaetigt: 5m 7.900 / 6,1m 9.700 / 7,3m 15.750 / 9,1m 18.000 EUR delivered+erected PT. Refs Brett (Quinta Glamping) + Paula Young (verkauft 7,3m gebraucht).</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
@@ -8277,7 +8277,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Quote schwach dokumentiert (kein IVA-Split, kein Quote-Nr, keine Bank), Klaerung gefordert</t>
+          <t>Nachfrage NIPC/IVA/Bankdaten/Material-Spec/Vermittlung Paula</t>
         </is>
       </c>
     </row>
@@ -8289,12 +8289,12 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Casa dos Sonhos (Sarah, PT)</t>
+          <t>Casa dos Sonhos (Sarah &amp; Vladimir, PT)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Facebook Messenger</t>
+          <t>PDF Quote</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -8304,128 +8304,128 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>SLOT OKTOBER 2026 ist an anderen Kunden vergeben. Naechster Slot 2027.</t>
-        </is>
-      </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>✗ Slot verloren</t>
+          <t>Quote 6,1m + 2.Tuer 850 + Flue-Kit 100 = 10.650 EUR. 1.000 EUR Anzahlung + 9.650 EUR am 1.8.2026. Lieferung 2. Oktoberwoche 2026.</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Quote erhalten</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Antwort raus: 2027er Slot + Preis-Bestaetigung + Paula-Vermittlung erfragen</t>
+          <t>Quote schwach dokumentiert (kein IVA-Split, kein Quote-Nr, keine Bank), Klaerung gefordert</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>~10.05.2026</t>
+          <t>15.05.2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Bēt Yurts (Noga &amp; Nadav, PT)</t>
+          <t>Casa dos Sonhos (Sarah, PT)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>E-Mail</t>
+          <t>Facebook Messenger</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Noga</t>
+          <t>Sarah -&gt; Sebastian</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Anfrage 6/7/9m Preise + Plattform + Aufbau Algarve</t>
-        </is>
-      </c>
-      <c r="F14" s="16" t="inlineStr">
-        <is>
-          <t>✓ Beantwortet</t>
+          <t>SLOT OKTOBER 2026 ist an anderen Kunden vergeben. Naechster Slot 2027.</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>✗ Slot verloren</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Antwort raus: 2027er Slot + Preis-Bestaetigung + Paula-Vermittlung erfragen</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>~12.05.2026</t>
+          <t>~10.05.2026</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Bēt Yurts (Noga, PT)</t>
+          <t>Bēt Yurts (Noga &amp; Nadav, PT)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>E-Mail + 3 PDF-Quotes</t>
+          <t>E-Mail</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Noga -&gt; Sebastian</t>
+          <t>Sebastian -&gt; Noga</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Preise: 6m=12.600 / 7m=14.400 / 9m=19.800 Jurte netto. Plattform separat: 6m=6.500 / 7m=7.200 / 9m=11.500. Transport+Install: 700/1.900, 900/2.500, 1.500/2.900. 23% IVA on top. 50% upfront NICHT-RUECKZAHLBAR. AUGUST 2026 Slot. Material laut Quote: Nordic Pine + Outer Canvas + 80mm Insulation (ohne Marken-Angabe). 2-J. Garantie auf Plane.</t>
+          <t>Anfrage 6/7/9m Preise + Plattform + Aufbau Algarve</t>
         </is>
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
-          <t>Quote erhalten</t>
+          <t>✓ Beantwortet</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Mail raus: Konkurrenz-Preis + Material-Aufschluesselung (Sauleda? PET?) anfordern</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>~17.05.2026</t>
+          <t>~12.05.2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Dune Algarve Sailmakers (PT)</t>
+          <t>Bēt Yurts (Noga, PT)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Web/E-Mail</t>
+          <t>E-Mail + 3 PDF-Quotes</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Dune</t>
+          <t>Noga -&gt; Sebastian</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Anfrage Sauleda-Plane 8m Massanfertigung</t>
-        </is>
-      </c>
-      <c r="F16" s="18" t="inlineStr">
-        <is>
-          <t>⏳ Antwort offen</t>
+          <t>Preise: 6m=12.600 / 7m=14.400 / 9m=19.800 Jurte netto. Plattform separat: 6m=6.500 / 7m=7.200 / 9m=11.500. Transport+Install: 700/1.900, 900/2.500, 1.500/2.900. 23% IVA on top. 50% upfront NICHT-RUECKZAHLBAR. AUGUST 2026 Slot. Material laut Quote: Nordic Pine + Outer Canvas + 80mm Insulation (ohne Marken-Angabe). 2-J. Garantie auf Plane.</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Quote erhalten</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>5 Tage warten, dann WhatsApp/Tel.-Nachfrage. Telefon-Skript bereit.</t>
+          <t>Mail raus: Konkurrenz-Preis + Material-Aufschluesselung (Sauleda? PET?) anfordern</t>
         </is>
       </c>
     </row>
@@ -8437,7 +8437,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Toldos Etapaveloz (Loule, PT)</t>
+          <t>Dune Algarve Sailmakers (PT)</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -8447,7 +8447,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Etapaveloz</t>
+          <t>Sebastian -&gt; Dune</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -8462,7 +8462,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>5 Tage warten, dann Folgekontakt</t>
+          <t>5 Tage warten, dann WhatsApp/Tel.-Nachfrage. Telefon-Skript bereit.</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Textilux (Algarve, PT)</t>
+          <t>Toldos Etapaveloz (Loule, PT)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -8484,7 +8484,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Textilux</t>
+          <t>Sebastian -&gt; Etapaveloz</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -8492,51 +8492,51 @@
           <t>Anfrage Sauleda-Plane 8m Massanfertigung</t>
         </is>
       </c>
-      <c r="F18" s="17" t="inlineStr">
-        <is>
-          <t>✗ ABGELEHNT</t>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>⏳ Antwort offen</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>'nao sao da nossa especialidade' - klassischer Markisen-Hersteller, kein 3D-Persenning. Keine weitere Aktion.</t>
+          <t>5 Tage warten, dann Folgekontakt</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>~17.05.2026</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Paula Young (FB 'Paula Vegan Chef')</t>
+          <t>Textilux (Algarve, PT)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Facebook (offen)</t>
+          <t>Web/E-Mail</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Paula</t>
+          <t>Sebastian -&gt; Textilux</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Anfrage zur gebrauchten 7,3m Casa-Jurte</t>
-        </is>
-      </c>
-      <c r="F19" s="18" t="inlineStr">
-        <is>
-          <t>⏳ Kontakt steht aus</t>
+          <t>Anfrage Sauleda-Plane 8m Massanfertigung</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>✗ ABGELEHNT</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Ueber FB suchen ODER Sarah um Vermittlung bitten (in der naechsten Casa-Antwort mit aufnehmen)</t>
+          <t>'nao sao da nossa especialidade' - klassischer Markisen-Hersteller, kein 3D-Persenning. Keine weitere Aktion.</t>
         </is>
       </c>
     </row>
@@ -8548,30 +8548,67 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
+          <t>Paula Young (FB 'Paula Vegan Chef')</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Facebook (offen)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Sebastian -&gt; Paula</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Anfrage zur gebrauchten 7,3m Casa-Jurte</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>⏳ Kontakt steht aus</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Ueber FB suchen ODER Sarah um Vermittlung bitten (in der naechsten Casa-Antwort mit aufnehmen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
           <t>Brett, Quinta Glamping (Algarve)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Online-Buchung</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Sebastian (geplant)</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Uebernachtung im Lake View Yurt (Casa dos Sonhos)</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F21" s="18" t="inlineStr">
         <is>
           <t>⏳ noch nicht gebucht</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Booking direkt: https://www.quintaglamping.com/rooms/lake-view-yurt.html - vor Anzahlung an Casa wertvoll</t>
         </is>

</xml_diff>

<commit_message>
Zwei neue Telegram-Kontakte: Mikael (8m-Angebot) + Dror (Experten-Ressource)
MIKAEL:
- Bietet komplette NEUE 8m Jurte, 2.10m Wandhoehe
- Sofort lieferbar, kann auch Massanfertigung
- Sebastian's Antwort raus: Standort? Preis? Cover-Material UV?
  Fotos? Hersteller oder privat?
- Wartet auf Specs+Preis

DROR (sehr wertvoll!):
- Stellt sich als Jurten-Experte vor (Bau+Reparatur)
- Bietet sich als Kontakt fuer Jurten-Fragen an
- Baut selbst (noch) keine Jurten
- Sebastian's Antwort raus: warmer Erstkontakt + Standort-Frage
- STRATEGIE: Sanity-Check vor Anzahlung Dani/Mikael/Benedikt,
  Material-Beurteilung, Plattform-Engineering Feedback

XLSX-Update:
- Sheet 15 (Kommunikations-Log): 4 neue Eintraege
- Mikael als potentielle 8m-Konkurrenz zu Benedikt 'Yury'
- Dror als unabhaengige Experten-Ressource fuer naechste Entscheidungen

https://claude.ai/code/session_01Wo6qsEhTrQuYRViomLojPq
</commit_message>
<xml_diff>
--- a/Jurten_Recherche_Algarve.xlsx
+++ b/Jurten_Recherche_Algarve.xlsx
@@ -8040,7 +8040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9429,67 +9429,215 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Sebastian -&gt; Selbst-Klaerung</t>
+          <t>Mikael (Telegram-Gruppe)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Analyse</t>
+          <t>Telegram-Post</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Intern</t>
+          <t>Mikael -&gt; Gruppe</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Frage 4cm Schafwolle Daemmung fuer Algarve-Winter ausreichend? Antwort: KNAPP. Dani's 4cm (R~1.05) ist halb so gut wie Bēt 8cm PET (R~2.1) und 1/3 vom DE-Niedrig-Bau-Standard. Aljezur-Atlantikkueste hat mildere Temperaturen als Castelo de Vide, aber starker Wind+Feuchtigkeit verstaerken Waermeverlust. MIT aktivem Holzofen+Top-Plattform-Daemmung (60-80mm Kork) = wohnen ja, mit Komfort-Limits. OHNE Heizen = nachts 8-12°C. DRINGEND: 8cm Upgrade bei Dani anfragen.</t>
+          <t>Bietet NEUE komplette 8m Jurte an, 2.10m Wandhoehe, sofort lieferbar, auch Massanfertigung anderer moeglich</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Analyse fertig</t>
+          <t>✓ Angebot erhalten</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Bei Dani 8cm Upgrade anfragen ODER Plattform-Daemmung als Kompensation auslegen (60-80mm Kork)</t>
+          <t>Sebastian -&gt; Mikael DM: Standort? Preis? Cover-Material UV? Fotos? Hersteller oder privat?</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
+          <t>23.05.2026</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Mikael (Telegram)</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Telegram DM</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Sebastian -&gt; Mikael</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Antwort kurz: 8m mit 2.10m Wand passt zu Plaenen Algarve. Frage: Standort? Preis? Cover-Material (UV-resistent?)? Fotos? Hersteller oder privat?</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>⏳ Zu senden</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Wartet auf Mikaels Antwort mit Specs+Preis</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>23.05.2026</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Dror (Telegram-Gruppe)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Telegram-Post</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Dror -&gt; Gruppe</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Stellt sich vor: viel Erfahrung im Jurten-BAU UND REPARATUR, baut selbst (noch) keine. Bietet sich als Kontakt fuer Jurten-Fragen an.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>✓ Wertvoller Kontakt</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Sebastian -&gt; Dror DM: warm danken, Projekt kurz erklaeren, signalisieren dass spaeter Sanity-Check kommen wird. Frage: Standort PT?</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>23.05.2026</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Dror (Telegram)</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Telegram DM</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Sebastian -&gt; Dror</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Warmer Erstkontakt: Vorstellung, Projekt-Beschreibung, signalisieren dass spaeter Sanity-Check kommt. Frage Standort PT.</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>⏳ Zu senden</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>DROR ALS WERTVOLLE RESSOURCE: Sanity-Check auf Dani/Benedikt/Mikael Angebote, Material-Beurteilung, Plattform-Engineering, Reparatur-Wissen fuer Zukunft. Konkrete Anfragen erst bei Auslosern (vor Anzahlung, vor Plattform-Bau, etc.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>23.05.2026</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Sebastian -&gt; Selbst-Klaerung</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Frage 4cm Schafwolle Daemmung fuer Algarve-Winter ausreichend? Antwort: KNAPP. Dani's 4cm (R~1.05) ist halb so gut wie Bēt 8cm PET (R~2.1) und 1/3 vom DE-Niedrig-Bau-Standard. Aljezur-Atlantikkueste hat mildere Temperaturen als Castelo de Vide, aber starker Wind+Feuchtigkeit verstaerken Waermeverlust. MIT aktivem Holzofen+Top-Plattform-Daemmung (60-80mm Kork) = wohnen ja, mit Komfort-Limits. OHNE Heizen = nachts 8-12°C. DRINGEND: 8cm Upgrade bei Dani anfragen.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Analyse fertig</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Bei Dani 8cm Upgrade anfragen ODER Plattform-Daemmung als Kompensation auslegen (60-80mm Kork)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>Brett, Quinta Glamping (Algarve)</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>Online-Buchung</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>Sebastian (geplant)</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>Uebernachtung im Lake View Yurt (Casa dos Sonhos)</t>
         </is>
       </c>
-      <c r="F39" s="19" t="inlineStr">
+      <c r="F43" s="19" t="inlineStr">
         <is>
           <t>⏳ noch nicht gebucht</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G43" s="3" t="inlineStr">
         <is>
           <t>Booking direkt: https://www.quintaglamping.com/rooms/lake-view-yurt.html - vor Anzahlung an Casa wertvoll</t>
         </is>

</xml_diff>

<commit_message>
Chris-Mail finalisiert: Aufbau-Frage konkretisierend statt offen
Sebastian-Feedback: Aufbau-Punkt umformuliert.
Statt 'wo findet der Aufbau statt' (offen, wirkt wie Sebastian
haette Danis frueheres 'inkl. Aufbau' nicht gehoert) jetzt
KONKRETISIEREND:

'Dani hatte gesagt, dass der Aufbau im Preis mit drin ist.
Wie darf ich mir das vorstellen? Liefert ihr direkt zu mir
nach Aljezur und baut dann vor Ort auf, oder laeuft das
anders?'

= signalisiert: Sebastian hat zugehoert, will jetzt Konkretes
verstehen. Respektiert Danis bisherige Aussagen.

REST DER MAIL UNVERAENDERT:
- Holz-Behandlung Termiten
- Plattform-Masse fuer DIY
- Lieferzeit Aug/Sep
- Probeschlafen-Termin

SCHAFWOLLE BEWUSST NICHT in dieser Mail (Sebastians Wunsch).
Kommt separat wenn Hauptklaerungen durch sind.

XLSX-Update:
- Sheet 15: Chris-Mail-Eintrag mit konkretisierter
  Aufbau-Frage dokumentiert

https://claude.ai/code/session_01Wo6qsEhTrQuYRViomLojPq
</commit_message>
<xml_diff>
--- a/Jurten_Recherche_Algarve.xlsx
+++ b/Jurten_Recherche_Algarve.xlsx
@@ -10407,7 +10407,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Persoenliche Einleitung + 4 inhaltliche Punkte (von urspruenglicher Dani-Mail): 1) Aufbau wo+Transport, 2) Holz-Behandlung Termiten, 3) Plattform-Masse fuer DIY, 4) Lieferzeit Aug/Sep konkret. PLUS integriert: Schafwoll-Frage (Chris ist Wolle-Quelle laut Dani). Plus Probeschlafen-Termin.</t>
+          <t>FINAL 4-Punkte-Mail an Chris: 1) AUFBAU - anerkennt Danis Aussage 'inkl. Aufbau', fragt KONKRETISIERUNG: liefert ihr zu mir nach Aljezur+Aufbau vor Ort? Transport extra/inkl? 2) Holz-Behandlung Termiten 3) Plattform-Masse fuer DIY 4) Lieferzeit Aug/Sep + Probeschlafen-Termin. Schafwoll-Frage bewusst NICHT in dieser Mail (kommt spaeter wenn naehere Klaerung).</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -10417,7 +10417,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>WICHTIGE KORREKTUR: Chris ist Danis Mann (Partner), nicht externer Anbieter! Sebastian schreibt direkt an ihn als technische Person des Paars. Beide getrennten Mails (Dani 4 Punkte + Chris Schafwoll) in EINE konsolidierte Chris-Mail integriert. Eine Person zu kontaktieren ist effizienter.</t>
+          <t>Persoenlich+praezise: 'Dani hatte gesagt' zeigt Sebastian geht nicht hinter Dani's Ruecken vorbei. Aufbau-Frage konkretisierend statt offen. 'euch' anerkennt Paar-Team.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dani-Antwort final: ESVO-Links direkt drin, demuetiger Teil raus
Sebastian-Anpassung:
- Konkrete ESVO-Links eingebaut (Sauleda + Boat-Canvas + Acrylic)
- Demuetigen 'Wartungs-Aufwand'-Schlussteil entfernt
- Klare, offensive Anfrage nach Premium-Material-Empfehlung

DREI ESVO-LINKS IN DER NACHRICHT:
- https://www.esvocampingshop.com/en/sauleda-en/
- https://www.esvocampingshop.com/en/tent-canvas/boat-canvas/
- https://www.esvocampingshop.com/en/tent-canvas/acrylic

XLSX-Update:
- Sheet 15: Sebastians finale Dani-Antwort mit ESVO-Links

NAECHSTE SCHRITTE:
- Antwort an Dani senden
- Auf Empfehlung warten (welche ESVO-Marine-Variante)
- Bei Empfehlung: Preis pruefen, Maschinen-Kompatibilitaet,
  finale Kalkulation Dani-Setup mit Marine-Plane

https://claude.ai/code/session_01Wo6qsEhTrQuYRViomLojPq
</commit_message>
<xml_diff>
--- a/Jurten_Recherche_Algarve.xlsx
+++ b/Jurten_Recherche_Algarve.xlsx
@@ -10637,7 +10637,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Begeistert: 'ESVO hat ja Sauleda und andere Marine-Acryl im Programm!' Sebastian schaut bei ESVO konkret. Vorschlag: Premium-Variante ueber Dani's gewohnten ESVO-Weg gehen (sie kennt Bestell-Prozedur, ESVO liefert kostenlos PT). Bittet Dani um EMPFEHLUNG welche ESVO-Marine-Variante fuer Algarve-Wohnjurte. Demuetig: 'falls ihr Sauleda nie genaeht habt, kein Druck - dann ESVO-Standard mit Wartung alle paar Jahre'.</t>
+          <t>Begeistert: 'ESVO hat ja Sauleda und andere Marine-Acryl im Programm!' Mit konkreten ESVO-Links (Sauleda + Boat-Canvas + Acrylic). Vorschlag: Premium-Variante ueber Danis gewohnten ESVO-Weg gehen (sie kennt Bestell-Prozedur, ESVO liefert kostenlos PT). Bittet Dani um EMPFEHLUNG welche ESVO-Marine-Variante fuer Algarve-Wohnjurte.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -10647,7 +10647,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Smart strategisch: Material-Wahl Dani uebergeben (sie kennt ESVO besser), Verantwortung Verarbeitung bei Dani. ESVO-Sauleda-Links als Verifikation.</t>
+          <t>Smart strategisch: Material-Wahl Dani uebergeben (sie kennt ESVO besser), Verantwortung Verarbeitung bei Dani. Direkte ESVO-Links als Verifikation. Demuetiger 'Wartungs-Aufwand'-Teil rausgenommen - klare offensive Botschaft.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mikael Option B FINAL Wording: ehrlich + Zeit-Bitte + freier Ausweg
https://claude.ai/code/session
</commit_message>
<xml_diff>
--- a/Jurten_Recherche_Algarve.xlsx
+++ b/Jurten_Recherche_Algarve.xlsx
@@ -11044,17 +11044,17 @@
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>OPTION B GEWAEHLT: Klare Linie - kein Geld vor Besuch. Ehrlich: 'cannot give full guarantee or any deposit before visit'. Akzeptiert wenn Mikael an anderen verkauft. Falls warten: Besuch 14/21 Juni, 5k sofort danach wenn alles wie beschrieben. Demuetig: 'whatever works for you - let me know honestly'.</t>
+          <t>OPTION B FINAL: 'I need a bit more time to make this decision. Big step for our family.' Verstaendnis fuer Mikaels Lage. Klare Ausweg-Option: 'if you can't wait, go ahead with another buyer - no hard feelings'. Falls warten: Besuch 14/21 Juni, 5k sofort danach. Demuetig + ehrlich: 'let me know honestly what works for you'.</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>⏳ Zu senden (Option B)</t>
+          <t>⏳ Zu senden</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>STRATEGISCHE BEDEUTUNG: Dani ist Sebastian's erste Wahl. Mikael ist akzeptables Verlustrisiko. Maximum Schutz. 3 mögliche Reaktionen: a) Ok ich warte bis Juni = Sebastian besucht beide. b) Doch 1-2k? = Nachverhandeln moeglich. c) Sorry muss verkaufen = Fokus voll auf Dani.</t>
+          <t>STRATEGIE: Sebastian will Zeit fuer Vergleich Dani vs Mikael. Maximum Ehrlichkeit + Akzeptanz Mikael verkauft. 3 mögliche Reaktionen: a) Mikael wartet = Sebastian besucht beide. b) Reservierungs-Verhandlung = Sebastian kann dann entscheiden. c) Mikael verkauft = Dani-Track fokussieren.</t>
         </is>
       </c>
     </row>

</xml_diff>